<commit_message>
historial y valores actualizados
</commit_message>
<xml_diff>
--- a/config/urls_scrapeo.xlsx
+++ b/config/urls_scrapeo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\The-Season\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26DBEC94-1DD3-43E9-B8F6-7BA0C774F0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481A8F95-B2A6-47E3-9455-8EA5FB8AE75C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$133</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -457,9 +457,6 @@
     <t>https://en.wikipedia.org/wiki/2020%E2%80%9321_Southern_Football_League#Premier_Division_Central</t>
   </si>
   <si>
-    <t>https://en.wikipedia.org/wiki/2019%E2%80%9320_Southern_Football_League#Premier_Division_Central</t>
-  </si>
-  <si>
     <t>https://en.wikipedia.org/wiki/2018%E2%80%9319_Southern_Football_League#Premier_Division_Central</t>
   </si>
   <si>
@@ -497,6 +494,9 @@
   </si>
   <si>
     <t>https://en.wikipedia.org/wiki/2015%E2%80%9316_Isthmian_League#Premier_Division</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/2018%E2%80%9320_Southern_Football_League#Premier_Division_Central</t>
   </si>
 </sst>
 </file>
@@ -845,7 +845,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:D133"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -868,7 +867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -882,7 +881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -896,7 +895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -910,7 +909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -924,7 +923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -938,7 +937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -952,7 +951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -966,7 +965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -980,7 +979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -994,7 +993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1016,13 +1015,13 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1036,7 +1035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -1050,7 +1049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1064,7 +1063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1078,7 +1077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -1092,7 +1091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1106,7 +1105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -1120,7 +1119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -1134,7 +1133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -1148,7 +1147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1170,13 +1169,13 @@
         <v>21</v>
       </c>
       <c r="C23" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D23">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -1190,7 +1189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -1204,7 +1203,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -1218,7 +1217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -1232,7 +1231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -1246,7 +1245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1260,7 +1259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>27</v>
       </c>
@@ -1274,7 +1273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>27</v>
       </c>
@@ -1288,7 +1287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>27</v>
       </c>
@@ -1296,13 +1295,13 @@
         <v>19</v>
       </c>
       <c r="C32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D32">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>27</v>
       </c>
@@ -1324,13 +1323,13 @@
         <v>21</v>
       </c>
       <c r="C34" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D34">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>32</v>
       </c>
@@ -1344,7 +1343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>32</v>
       </c>
@@ -1358,7 +1357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>32</v>
       </c>
@@ -1372,7 +1371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>32</v>
       </c>
@@ -1386,7 +1385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -1400,7 +1399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>32</v>
       </c>
@@ -1414,7 +1413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>32</v>
       </c>
@@ -1428,7 +1427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>32</v>
       </c>
@@ -1442,21 +1441,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>32</v>
       </c>
       <c r="B43" t="s">
         <v>19</v>
       </c>
-      <c r="C43" t="s">
-        <v>144</v>
+      <c r="C43" s="1" t="s">
+        <v>157</v>
       </c>
       <c r="D43">
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>32</v>
       </c>
@@ -1478,13 +1477,13 @@
         <v>21</v>
       </c>
       <c r="C45" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D45">
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>37</v>
       </c>
@@ -1498,7 +1497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>37</v>
       </c>
@@ -1512,7 +1511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>37</v>
       </c>
@@ -1526,7 +1525,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>37</v>
       </c>
@@ -1540,7 +1539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>37</v>
       </c>
@@ -1554,7 +1553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>37</v>
       </c>
@@ -1568,7 +1567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>37</v>
       </c>
@@ -1582,7 +1581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>37</v>
       </c>
@@ -1596,7 +1595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>37</v>
       </c>
@@ -1610,7 +1609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>37</v>
       </c>
@@ -1632,13 +1631,13 @@
         <v>21</v>
       </c>
       <c r="C56" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D56">
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>42</v>
       </c>
@@ -1652,7 +1651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>42</v>
       </c>
@@ -1666,7 +1665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>42</v>
       </c>
@@ -1680,7 +1679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>42</v>
       </c>
@@ -1694,7 +1693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>42</v>
       </c>
@@ -1708,7 +1707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>42</v>
       </c>
@@ -1722,7 +1721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>42</v>
       </c>
@@ -1736,7 +1735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>42</v>
       </c>
@@ -1750,7 +1749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>42</v>
       </c>
@@ -1764,7 +1763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>42</v>
       </c>
@@ -1786,13 +1785,13 @@
         <v>21</v>
       </c>
       <c r="C67" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D67">
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>47</v>
       </c>
@@ -1806,7 +1805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>47</v>
       </c>
@@ -1820,7 +1819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>47</v>
       </c>
@@ -1834,7 +1833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>47</v>
       </c>
@@ -1848,7 +1847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>47</v>
       </c>
@@ -1862,7 +1861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>47</v>
       </c>
@@ -1876,7 +1875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>47</v>
       </c>
@@ -1890,7 +1889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>47</v>
       </c>
@@ -1904,7 +1903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>47</v>
       </c>
@@ -1918,7 +1917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>47</v>
       </c>
@@ -1940,13 +1939,13 @@
         <v>21</v>
       </c>
       <c r="C78" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D78">
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>52</v>
       </c>
@@ -1960,7 +1959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>52</v>
       </c>
@@ -1974,7 +1973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>52</v>
       </c>
@@ -1988,7 +1987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>52</v>
       </c>
@@ -2002,7 +2001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>52</v>
       </c>
@@ -2016,7 +2015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>52</v>
       </c>
@@ -2030,7 +2029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>52</v>
       </c>
@@ -2044,7 +2043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>52</v>
       </c>
@@ -2058,7 +2057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>52</v>
       </c>
@@ -2072,7 +2071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>52</v>
       </c>
@@ -2094,13 +2093,13 @@
         <v>21</v>
       </c>
       <c r="C89" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D89">
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>57</v>
       </c>
@@ -2114,7 +2113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>57</v>
       </c>
@@ -2128,7 +2127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>57</v>
       </c>
@@ -2142,7 +2141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>57</v>
       </c>
@@ -2156,7 +2155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>57</v>
       </c>
@@ -2170,7 +2169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>57</v>
       </c>
@@ -2184,7 +2183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>57</v>
       </c>
@@ -2198,7 +2197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>57</v>
       </c>
@@ -2212,7 +2211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>57</v>
       </c>
@@ -2226,7 +2225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>57</v>
       </c>
@@ -2248,13 +2247,13 @@
         <v>21</v>
       </c>
       <c r="C100" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D100">
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>62</v>
       </c>
@@ -2268,7 +2267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>62</v>
       </c>
@@ -2282,7 +2281,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>62</v>
       </c>
@@ -2296,7 +2295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>62</v>
       </c>
@@ -2310,7 +2309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>62</v>
       </c>
@@ -2324,7 +2323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>62</v>
       </c>
@@ -2338,7 +2337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>62</v>
       </c>
@@ -2352,7 +2351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>62</v>
       </c>
@@ -2366,7 +2365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>62</v>
       </c>
@@ -2380,7 +2379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>62</v>
       </c>
@@ -2402,13 +2401,13 @@
         <v>21</v>
       </c>
       <c r="C111" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D111">
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>67</v>
       </c>
@@ -2422,7 +2421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>67</v>
       </c>
@@ -2436,7 +2435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>67</v>
       </c>
@@ -2450,7 +2449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>67</v>
       </c>
@@ -2464,7 +2463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>67</v>
       </c>
@@ -2478,7 +2477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>67</v>
       </c>
@@ -2492,7 +2491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>67</v>
       </c>
@@ -2506,7 +2505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>67</v>
       </c>
@@ -2520,7 +2519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>67</v>
       </c>
@@ -2534,7 +2533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>67</v>
       </c>
@@ -2556,13 +2555,13 @@
         <v>21</v>
       </c>
       <c r="C122" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D122">
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>103</v>
       </c>
@@ -2576,7 +2575,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>103</v>
       </c>
@@ -2590,7 +2589,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>103</v>
       </c>
@@ -2604,7 +2603,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="126" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>103</v>
       </c>
@@ -2618,7 +2617,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>103</v>
       </c>
@@ -2632,7 +2631,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>103</v>
       </c>
@@ -2646,7 +2645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>103</v>
       </c>
@@ -2660,7 +2659,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>103</v>
       </c>
@@ -2674,7 +2673,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>103</v>
       </c>
@@ -2688,7 +2687,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="132" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>103</v>
       </c>
@@ -2710,20 +2709,14 @@
         <v>21</v>
       </c>
       <c r="C133" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D133">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D132" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Isthmian League Premier Division"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:D133" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="C17" r:id="rId1" xr:uid="{E1B85167-3D2A-42BA-99C6-C7D7ED1D704A}"/>
     <hyperlink ref="C128" r:id="rId2" location="National_League_North" xr:uid="{D73DF404-E92B-4233-877F-1853371C40E1}"/>
@@ -2733,8 +2726,9 @@
     <hyperlink ref="C11" r:id="rId6" location="Premier_Division_South" xr:uid="{C60537E5-0463-446C-A564-7243F1667314}"/>
     <hyperlink ref="C131" r:id="rId7" location="Premier_Division_South" xr:uid="{10A11A83-8674-49EB-AE69-E25F907A25CE}"/>
     <hyperlink ref="C132" r:id="rId8" location="Premier_Division_Central" xr:uid="{62C11DCC-7435-446A-909D-4DB76DA847AC}"/>
+    <hyperlink ref="C43" r:id="rId9" location="Premier_Division_Central" xr:uid="{0E67DA2E-055C-46F2-84E9-D99C4D71B1C1}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId9"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
reglamento y valores actualizados
</commit_message>
<xml_diff>
--- a/config/urls_scrapeo.xlsx
+++ b/config/urls_scrapeo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\The-Season\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481A8F95-B2A6-47E3-9455-8EA5FB8AE75C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F1D9B0-8B82-4DBC-A166-0A24F1DE7DD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -845,6 +845,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D133"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -867,7 +868,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -881,7 +882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -895,7 +896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -909,7 +910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -923,7 +924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -937,7 +938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -951,7 +952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -965,7 +966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -979,7 +980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -993,7 +994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1007,7 +1008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1175,7 +1176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -1189,7 +1190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -1203,7 +1204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -1217,7 +1218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -1231,7 +1232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -1245,7 +1246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1259,7 +1260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>27</v>
       </c>
@@ -1273,7 +1274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>27</v>
       </c>
@@ -1287,7 +1288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>27</v>
       </c>
@@ -1301,7 +1302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>27</v>
       </c>
@@ -1315,7 +1316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -1329,7 +1330,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>32</v>
       </c>
@@ -1343,7 +1344,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>32</v>
       </c>
@@ -1357,7 +1358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>32</v>
       </c>
@@ -1371,7 +1372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>32</v>
       </c>
@@ -1385,7 +1386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -1399,7 +1400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>32</v>
       </c>
@@ -1413,7 +1414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>32</v>
       </c>
@@ -1427,7 +1428,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>32</v>
       </c>
@@ -1441,7 +1442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>32</v>
       </c>
@@ -1455,7 +1456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>32</v>
       </c>
@@ -1469,7 +1470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>32</v>
       </c>
@@ -1483,7 +1484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>37</v>
       </c>
@@ -1497,7 +1498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>37</v>
       </c>
@@ -1511,7 +1512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>37</v>
       </c>
@@ -1525,7 +1526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>37</v>
       </c>
@@ -1539,7 +1540,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>37</v>
       </c>
@@ -1553,7 +1554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>37</v>
       </c>
@@ -1567,7 +1568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>37</v>
       </c>
@@ -1581,7 +1582,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>37</v>
       </c>
@@ -1595,7 +1596,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>37</v>
       </c>
@@ -1609,7 +1610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>37</v>
       </c>
@@ -1623,7 +1624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>37</v>
       </c>
@@ -1637,7 +1638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>42</v>
       </c>
@@ -1651,7 +1652,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>42</v>
       </c>
@@ -1665,7 +1666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>42</v>
       </c>
@@ -1679,7 +1680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>42</v>
       </c>
@@ -1693,7 +1694,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>42</v>
       </c>
@@ -1707,7 +1708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>42</v>
       </c>
@@ -1721,7 +1722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>42</v>
       </c>
@@ -1735,7 +1736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>42</v>
       </c>
@@ -1749,7 +1750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>42</v>
       </c>
@@ -1763,7 +1764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>42</v>
       </c>
@@ -1777,7 +1778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>42</v>
       </c>
@@ -1791,7 +1792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>47</v>
       </c>
@@ -1805,7 +1806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>47</v>
       </c>
@@ -1819,7 +1820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>47</v>
       </c>
@@ -1833,7 +1834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>47</v>
       </c>
@@ -1847,7 +1848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>47</v>
       </c>
@@ -1861,7 +1862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>47</v>
       </c>
@@ -1875,7 +1876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>47</v>
       </c>
@@ -1889,7 +1890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>47</v>
       </c>
@@ -1903,7 +1904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>47</v>
       </c>
@@ -1917,7 +1918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>47</v>
       </c>
@@ -1931,7 +1932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>47</v>
       </c>
@@ -1945,7 +1946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>52</v>
       </c>
@@ -1959,7 +1960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>52</v>
       </c>
@@ -1973,7 +1974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>52</v>
       </c>
@@ -1987,7 +1988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>52</v>
       </c>
@@ -2001,7 +2002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>52</v>
       </c>
@@ -2015,7 +2016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>52</v>
       </c>
@@ -2029,7 +2030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>52</v>
       </c>
@@ -2043,7 +2044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>52</v>
       </c>
@@ -2057,7 +2058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>52</v>
       </c>
@@ -2071,7 +2072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>52</v>
       </c>
@@ -2085,7 +2086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>52</v>
       </c>
@@ -2099,7 +2100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>57</v>
       </c>
@@ -2113,7 +2114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>57</v>
       </c>
@@ -2127,7 +2128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>57</v>
       </c>
@@ -2141,7 +2142,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>57</v>
       </c>
@@ -2155,7 +2156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>57</v>
       </c>
@@ -2169,7 +2170,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>57</v>
       </c>
@@ -2183,7 +2184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>57</v>
       </c>
@@ -2197,7 +2198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>57</v>
       </c>
@@ -2211,7 +2212,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>57</v>
       </c>
@@ -2225,7 +2226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>57</v>
       </c>
@@ -2239,7 +2240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>57</v>
       </c>
@@ -2253,7 +2254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>62</v>
       </c>
@@ -2267,7 +2268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>62</v>
       </c>
@@ -2281,7 +2282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>62</v>
       </c>
@@ -2295,7 +2296,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>62</v>
       </c>
@@ -2309,7 +2310,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>62</v>
       </c>
@@ -2323,7 +2324,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>62</v>
       </c>
@@ -2337,7 +2338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>62</v>
       </c>
@@ -2351,7 +2352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>62</v>
       </c>
@@ -2365,7 +2366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>62</v>
       </c>
@@ -2379,7 +2380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>62</v>
       </c>
@@ -2393,7 +2394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>62</v>
       </c>
@@ -2407,7 +2408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>67</v>
       </c>
@@ -2421,7 +2422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>67</v>
       </c>
@@ -2435,7 +2436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>67</v>
       </c>
@@ -2449,7 +2450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>67</v>
       </c>
@@ -2463,7 +2464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>67</v>
       </c>
@@ -2477,7 +2478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>67</v>
       </c>
@@ -2491,7 +2492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>67</v>
       </c>
@@ -2505,7 +2506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>67</v>
       </c>
@@ -2519,7 +2520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>67</v>
       </c>
@@ -2533,7 +2534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>67</v>
       </c>
@@ -2547,7 +2548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>67</v>
       </c>
@@ -2561,7 +2562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>103</v>
       </c>
@@ -2575,7 +2576,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>103</v>
       </c>
@@ -2589,7 +2590,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>103</v>
       </c>
@@ -2603,7 +2604,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>103</v>
       </c>
@@ -2617,7 +2618,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>103</v>
       </c>
@@ -2631,7 +2632,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>103</v>
       </c>
@@ -2645,7 +2646,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>103</v>
       </c>
@@ -2659,7 +2660,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>103</v>
       </c>
@@ -2673,7 +2674,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>103</v>
       </c>
@@ -2687,7 +2688,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>103</v>
       </c>
@@ -2701,7 +2702,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>103</v>
       </c>
@@ -2716,7 +2717,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D133" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:D133" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="2016/17"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="C17" r:id="rId1" xr:uid="{E1B85167-3D2A-42BA-99C6-C7D7ED1D704A}"/>
     <hyperlink ref="C128" r:id="rId2" location="National_League_North" xr:uid="{D73DF404-E92B-4233-877F-1853371C40E1}"/>

</xml_diff>